<commit_message>
General improvements to ODM v2 ID code
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/nwss-reporting-to-v2/ids/general_v2_id_code.xlsx
+++ b/odm_map/data/modules/nwss-reporting-to-v2/ids/general_v2_id_code.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/nwss-reporting-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1BC612-576A-2847-B4A0-819BC7F8F3F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638F6E2D-9375-B04D-AB5F-D9C3F40BFEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="95">
   <si>
     <t>addresses</t>
   </si>
@@ -175,30 +175,15 @@
     <t>fn.makeid(datEmpty.qualityReports.qualityFlag, datEmpty.qualityReports.measureRepID if datEmpty.qualityReports.__measureRepID else datEmpty.qualityReports.sampleID if datEmpty.qualityReports.__sampleID else datEmpty.qualityReports.measureSetRepID)</t>
   </si>
   <si>
-    <t>dat.addresses.__addressID</t>
-  </si>
-  <si>
     <t>dat.datasets.datasetID</t>
   </si>
   <si>
-    <t>dat.contacts.__contactID</t>
-  </si>
-  <si>
     <t>dat.organizations.organizationID</t>
   </si>
   <si>
-    <t>dat.datasets.__datasetID</t>
-  </si>
-  <si>
-    <t>dat.instruments.__instrumentID</t>
-  </si>
-  <si>
     <t>dat.contacts.contactID</t>
   </si>
   <si>
-    <t>dat.measures.__measureRepID</t>
-  </si>
-  <si>
     <t>dat.protocols.protocolID</t>
   </si>
   <si>
@@ -214,18 +199,9 @@
     <t>dat.measureSets.measureSetRepID</t>
   </si>
   <si>
-    <t>dat.organizations.__organizationID</t>
-  </si>
-  <si>
     <t>dat.addresses.addressID</t>
   </si>
   <si>
-    <t>dat.polygons.__polygonID</t>
-  </si>
-  <si>
-    <t>dat.protocols.__protocolID</t>
-  </si>
-  <si>
     <t>dat.instruments.instrumentID</t>
   </si>
   <si>
@@ -238,12 +214,6 @@
     <t>dat.measureSets.measureSetRepID if dat.qualityReports.__measureSetRepID else ""</t>
   </si>
   <si>
-    <t>dat.samples.__sampleID</t>
-  </si>
-  <si>
-    <t>dat.sites.__siteID</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3])</t>
   </si>
   <si>
@@ -289,9 +259,6 @@
     <t>fn.makeid(datEmpty.samples.siteID, datEmpty.samples.collDT if dat.samples.collDT else datEmpty.samples.collDTEnd, f"{fn.rownum:03d}")</t>
   </si>
   <si>
-    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "(__source_file_and_row__)", equals=dat.measureSets.get("(__source_file_and_row__)"))))</t>
-  </si>
-  <si>
     <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
   </si>
   <si>
@@ -314,6 +281,45 @@
   </si>
   <si>
     <t>fn.datetimetz(dat.samples.__collDTEnd.split('/!/'))</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.sites.__siteID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.samples.__sampleID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.addresses.__addressID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.contacts.__contactID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.datasets.__datasetID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.instruments.__instrumentID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.measures.__measureRepID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.organizations.__organizationID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.polygons.__polygonID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.protocols.__protocolID)</t>
+  </si>
+  <si>
+    <t>datEmpty.organizations.organizationID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures")))</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, dat.qualityReports.measureRepID, dat.qualityReports.sampleID, dat.qualityReports.measureSetRepID)</t>
   </si>
 </sst>
 </file>
@@ -705,13 +711,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -722,7 +728,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -733,10 +739,10 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -747,7 +753,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -758,7 +764,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -782,10 +788,10 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -828,13 +834,13 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -845,7 +851,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -856,7 +862,7 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -867,7 +873,7 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -883,13 +889,13 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E25" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -900,7 +906,7 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -911,7 +917,7 @@
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -922,7 +928,7 @@
         <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -933,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -944,7 +950,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -955,7 +961,7 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -966,7 +972,7 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -977,7 +983,7 @@
         <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -988,10 +994,10 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="E35" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1002,7 +1008,7 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1013,7 +1019,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1024,7 +1030,7 @@
         <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1035,10 +1041,10 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1049,7 +1055,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1060,7 +1066,7 @@
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1071,13 +1077,13 @@
         <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E44" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1088,7 +1094,7 @@
         <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1099,7 +1105,7 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1110,7 +1116,7 @@
         <v>11</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1118,10 +1124,10 @@
         <v>37</v>
       </c>
       <c r="B49" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="C49" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1140,10 +1146,10 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="D52" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1154,7 +1160,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1165,7 +1171,7 @@
         <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1176,7 +1182,7 @@
         <v>11</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1187,7 +1193,7 @@
         <v>15</v>
       </c>
       <c r="C57" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1198,7 +1204,7 @@
         <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -1209,7 +1215,7 @@
         <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -1220,7 +1226,7 @@
         <v>16</v>
       </c>
       <c r="C60" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
@@ -1231,6 +1237,9 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
+        <v>94</v>
+      </c>
+      <c r="E62" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1242,10 +1251,10 @@
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E63" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -1255,8 +1264,11 @@
       <c r="B64" t="s">
         <v>6</v>
       </c>
+      <c r="C64" t="s">
+        <v>50</v>
+      </c>
       <c r="E64" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
@@ -1266,8 +1278,11 @@
       <c r="B65" t="s">
         <v>9</v>
       </c>
+      <c r="C65" t="s">
+        <v>53</v>
+      </c>
       <c r="E65" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -1283,10 +1298,10 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="D69" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -1297,7 +1312,7 @@
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -1308,7 +1323,7 @@
         <v>10</v>
       </c>
       <c r="C71" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
@@ -1319,7 +1334,7 @@
         <v>11</v>
       </c>
       <c r="C72" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
@@ -1330,7 +1345,7 @@
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -1341,7 +1356,7 @@
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -1349,10 +1364,10 @@
         <v>19</v>
       </c>
       <c r="B75" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C75" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1360,10 +1375,10 @@
         <v>19</v>
       </c>
       <c r="B76" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C76" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -1371,10 +1386,10 @@
         <v>19</v>
       </c>
       <c r="B77" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C77" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -1393,10 +1408,10 @@
         <v>8</v>
       </c>
       <c r="C80" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="D80" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -1407,7 +1422,7 @@
         <v>2</v>
       </c>
       <c r="C81" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
@@ -1418,7 +1433,7 @@
         <v>7</v>
       </c>
       <c r="C82" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
@@ -1429,7 +1444,7 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -1440,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="C84" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -1451,7 +1466,7 @@
         <v>11</v>
       </c>
       <c r="C85" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>